<commit_message>
Fix Phase 4: remove op_r from ALU case selection to prevent instruction corruption
The op_r mechanism held the previous MUL/DIV opcode for one extra cycle,
causing every instruction immediately following a MUL/DIV to compute
with the wrong ALU operation. Since the combinational ALU (busy=0)
completes all operations in one cycle, op_r-based selection is dead code
that only causes harm. Changed `case (op_r != 0 ? op_r : op)` to `case (op)`.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datapath_control_table_miniRV.xlsx
+++ b/datapath_control_table_miniRV.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HuaweiMoveData\Users\20805\Desktop\homework\CPU_lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_5393FADBEB04207D84E0239C90DFEE2AF7CF8380" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA2A70F1-F18B-404A-9922-F7BA69800F8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="14595" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="14595" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="数据通路表(含控制信号)" sheetId="1" r:id="rId1"/>
@@ -743,21 +743,21 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1065,96 +1065,103 @@
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="6" width="6" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" customWidth="1"/>
+    <col min="4" max="4" width="6" customWidth="1"/>
+    <col min="5" max="5" width="11.86328125" customWidth="1"/>
+    <col min="6" max="6" width="21.53125" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="10" width="8" customWidth="1"/>
+    <col min="8" max="8" width="13.33203125" customWidth="1"/>
+    <col min="9" max="9" width="14.9296875" customWidth="1"/>
+    <col min="10" max="10" width="8" customWidth="1"/>
     <col min="11" max="11" width="24" customWidth="1"/>
-    <col min="12" max="12" width="6" customWidth="1"/>
-    <col min="13" max="15" width="8" customWidth="1"/>
+    <col min="12" max="12" width="10.265625" customWidth="1"/>
+    <col min="13" max="13" width="12.73046875" customWidth="1"/>
+    <col min="14" max="14" width="14.46484375" customWidth="1"/>
+    <col min="15" max="15" width="8" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
     <col min="17" max="17" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:17" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="12"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10"/>
     </row>
     <row r="2" spans="2:17" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:17" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="9" t="s">
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="9" t="s">
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="M3" s="12"/>
-      <c r="N3" s="9" t="s">
+      <c r="M3" s="10"/>
+      <c r="N3" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
     </row>
     <row r="4" spans="2:17" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="9" t="s">
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="10"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="15"/>
       <c r="K4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="L4" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="M4" s="10"/>
-      <c r="N4" s="9" t="s">
+      <c r="M4" s="15"/>
+      <c r="N4" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="O4" s="10"/>
-      <c r="P4" s="9" t="s">
+      <c r="O4" s="15"/>
+      <c r="P4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="Q4" s="10"/>
+      <c r="Q4" s="15"/>
     </row>
     <row r="5" spans="2:17" ht="20" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="2"/>
@@ -1705,84 +1712,84 @@
       </c>
     </row>
     <row r="18" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="12"/>
-      <c r="M18" s="12"/>
-      <c r="N18" s="12"/>
-      <c r="O18" s="12"/>
-      <c r="P18" s="12"/>
-      <c r="Q18" s="12"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="10"/>
     </row>
     <row r="19" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="9" t="s">
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="9" t="s">
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="M19" s="12"/>
-      <c r="N19" s="9" t="s">
+      <c r="M19" s="10"/>
+      <c r="N19" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="O19" s="12"/>
-      <c r="P19" s="12"/>
-      <c r="Q19" s="12"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10"/>
     </row>
     <row r="20" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="9" t="s">
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="10"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="15"/>
       <c r="K20" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L20" s="9" t="s">
+      <c r="L20" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="M20" s="10"/>
-      <c r="N20" s="9" t="s">
+      <c r="M20" s="15"/>
+      <c r="N20" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="O20" s="10"/>
-      <c r="P20" s="9" t="s">
+      <c r="O20" s="15"/>
+      <c r="P20" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="Q20" s="10"/>
+      <c r="Q20" s="15"/>
     </row>
     <row r="21" spans="2:17" ht="22.5" x14ac:dyDescent="0.3">
       <c r="B21" s="2"/>
@@ -3734,6 +3741,12 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="P20:Q20"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="L20:M20"/>
     <mergeCell ref="C20:F20"/>
     <mergeCell ref="N3:Q3"/>
     <mergeCell ref="B1:Q1"/>
@@ -3750,12 +3763,6 @@
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="B18:Q18"/>
     <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="P20:Q20"/>
-    <mergeCell ref="G4:J4"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="L20:M20"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3776,49 +3783,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
     </row>
     <row r="2" spans="2:15" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="9" t="s">
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="G3" s="12"/>
-      <c r="H3" s="9" t="s">
+      <c r="G3" s="10"/>
+      <c r="H3" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
       <c r="K3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="L3" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="M3" s="12"/>
+      <c r="M3" s="10"/>
       <c r="N3" s="1" t="s">
         <v>108</v>
       </c>
@@ -4221,48 +4228,48 @@
       </c>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="12"/>
-      <c r="M14" s="12"/>
-      <c r="N14" s="12"/>
-      <c r="O14" s="12"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="9" t="s">
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="G15" s="12"/>
-      <c r="H15" s="9" t="s">
+      <c r="G15" s="10"/>
+      <c r="H15" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
       <c r="K15" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L15" s="9" t="s">
+      <c r="L15" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="M15" s="12"/>
+      <c r="M15" s="10"/>
       <c r="N15" s="1" t="s">
         <v>108</v>
       </c>
@@ -5897,25 +5904,28 @@
       </c>
     </row>
     <row r="55" spans="2:15" x14ac:dyDescent="0.3">
-      <c r="B55" s="15" t="s">
+      <c r="B55" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="C55" s="12"/>
-      <c r="D55" s="12"/>
-      <c r="E55" s="12"/>
-      <c r="F55" s="12"/>
-      <c r="G55" s="12"/>
-      <c r="H55" s="12"/>
-      <c r="I55" s="12"/>
-      <c r="J55" s="12"/>
-      <c r="K55" s="12"/>
-      <c r="L55" s="12"/>
-      <c r="M55" s="12"/>
-      <c r="N55" s="12"/>
-      <c r="O55" s="12"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="10"/>
+      <c r="E55" s="10"/>
+      <c r="F55" s="10"/>
+      <c r="G55" s="10"/>
+      <c r="H55" s="10"/>
+      <c r="I55" s="10"/>
+      <c r="J55" s="10"/>
+      <c r="K55" s="10"/>
+      <c r="L55" s="10"/>
+      <c r="M55" s="10"/>
+      <c r="N55" s="10"/>
+      <c r="O55" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B1:O1"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="F15:G15"/>
     <mergeCell ref="B55:O55"/>
     <mergeCell ref="L15:M15"/>
     <mergeCell ref="C3:E3"/>
@@ -5924,9 +5934,6 @@
     <mergeCell ref="B14:O14"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="L3:M3"/>
-    <mergeCell ref="B1:O1"/>
-    <mergeCell ref="H15:J15"/>
-    <mergeCell ref="F15:G15"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>